<commit_message>
Fix Milestone 2 feedback and document deferred GUI work
</commit_message>
<xml_diff>
--- a/Milestone 2/UVSim-Milestone-2-Unit-Tests.xlsx
+++ b/Milestone 2/UVSim-Milestone-2-Unit-Tests.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit tests" sheetId="1" r:id="R1847477327704d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit tests" sheetId="1" r:id="R35222bd540c6423c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -38,6 +38,11 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF243746"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -70,7 +75,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -107,6 +112,13 @@
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -115,7 +127,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UnitTestRegister" displayName="UnitTestRegister" ref="A8:H41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="UnitTestRegister" displayName="UnitTestRegister" ref="A8:H44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Test name"/>
@@ -350,7 +362,7 @@
     </x:row>
     <x:row r="2" ht="29" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>UVSim milestone 2 — unit test register</x:v>
+        <x:v>UVSim - console feedback revision test register</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -362,7 +374,7 @@
     </x:row>
     <x:row r="3" ht="21" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>Source: main (37e2789); 33 test methods. Use-case IDs follow docs/design.md.</x:v>
+        <x:v>36 test methods. Use-case IDs match Milestone 2/design.md and the revised PDF. GUI recovery is deferred.</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -398,7 +410,7 @@
     </x:row>
     <x:row r="6" ht="21" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>Criteria describe expected behavior, not a recorded execution result. UC-14 row covers the HALT handler only.</x:v>
+        <x:v>Expected criteria, not recorded execution results. UT-33 covers HALT directly; UT-34 covers console execution.</x:v>
       </x:c>
       <x:c r="B6" s="3"/>
       <x:c r="C6" s="3"/>
@@ -995,22 +1007,22 @@
         <x:v>UT-22</x:v>
       </x:c>
       <x:c r="B30" s="14" t="str">
-        <x:v>test_overflow_preserves_accumulator</x:v>
+        <x:v>test_overflow_truncates_and_preserves_sign</x:v>
       </x:c>
       <x:c r="C30" s="14" t="str">
         <x:v>UC-07, UC-08, UC-10</x:v>
       </x:c>
       <x:c r="D30" s="14" t="str">
-        <x:v>Reject arithmetic overflow at both word limits.</x:v>
+        <x:v>Truncate overflow magnitude and retain sign.</x:v>
       </x:c>
       <x:c r="E30" s="14" t="str">
-        <x:v>ADD: (9999, 1), (-9999, -1). SUBTRACT: (-9999, 1), (9999, -1). MULTIPLY: (9999, 2), (-9999, 2). Pairs are accumulator and memory[42].</x:v>
+        <x:v>ADD/SUB: +/-10000; MULTIPLY: +/-19998, +/-12345, 9999*9999.</x:v>
       </x:c>
       <x:c r="F30" s="14" t="str">
-        <x:v>ValueError containing "between -9999 and 9999"; original accumulator preserved.</x:v>
+        <x:v>Results: 0, +/-9998, +/-2345, 1.</x:v>
       </x:c>
       <x:c r="G30" s="14" t="str">
-        <x:v>Pass if the expected error and unchanged accumulator hold in all six subcases.</x:v>
+        <x:v>Pass if all nine subcases match without overflow errors.</x:v>
       </x:c>
       <x:c r="H30" s="14" t="str">
         <x:v>tests/test_arithmetic.py</x:v>
@@ -1082,7 +1094,7 @@
         <x:v>Verify arithmetic dispatch mapping at addresses 00 and 99.</x:v>
       </x:c>
       <x:c r="E33" s="13" t="str">
-        <x:v>Accumulator 12; operand memory 3. Opcodes 30–33 at addresses 0 and 99. Counter 8; register = opcode * 100 + address; halted False.</x:v>
+        <x:v>Accumulator 12; operand memory 3. Opcodes 30-33 at addresses 0 and 99. Counter 8; register = opcode * 100 + address; halted False.</x:v>
       </x:c>
       <x:c r="F33" s="13" t="str">
         <x:v>Results: 30 = 15, 31 = 9, 32 = 4, 33 = 36. Memory, counter, register and halted state unchanged.</x:v>
@@ -1302,10 +1314,88 @@
         <x:v>tests/test_control_flow.py</x:v>
       </x:c>
     </x:row>
+    <x:row r="42" ht="100" customHeight="1">
+      <x:c r="A42" s="18" t="str">
+        <x:v>UT-34</x:v>
+      </x:c>
+      <x:c r="B42" s="18" t="str">
+        <x:v>test_instructor_programs</x:v>
+      </x:c>
+      <x:c r="C42" s="18" t="str">
+        <x:v>UC-01, UC-03, UC-04, UC-07, UC-08, UC-09, UC-10, UC-11, UC-12, UC-13, UC-14</x:v>
+      </x:c>
+      <x:c r="D42" s="18" t="str">
+        <x:v>Execute supplied programs using console I/O.</x:v>
+      </x:c>
+      <x:c r="E42" s="18" t="str">
+        <x:v>Test1 7,5; Test2 both orders/equal/negative; Test3/3b/4 no input.</x:v>
+      </x:c>
+      <x:c r="F42" s="18" t="str">
+        <x:v>Expected milestone numeric sequences and HALT.</x:v>
+      </x:c>
+      <x:c r="G42" s="18" t="str">
+        <x:v>Pass if all eight cases halt and output matches.</x:v>
+      </x:c>
+      <x:c r="H42" s="18" t="str">
+        <x:v>tests/test_regression.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="100" customHeight="1">
+      <x:c r="A43" s="18" t="str">
+        <x:v>UT-35</x:v>
+      </x:c>
+      <x:c r="B43" s="18" t="str">
+        <x:v>test_write_four_digits_and_negative_sign</x:v>
+      </x:c>
+      <x:c r="C43" s="18" t="str">
+        <x:v>UC-04</x:v>
+      </x:c>
+      <x:c r="D43" s="18" t="str">
+        <x:v>Format four magnitude digits.</x:v>
+      </x:c>
+      <x:c r="E43" s="18" t="str">
+        <x:v>1234,12,0,-5,-9999.</x:v>
+      </x:c>
+      <x:c r="F43" s="18" t="str">
+        <x:v>1234,0012,0000,-0005,-9999.</x:v>
+      </x:c>
+      <x:c r="G43" s="18" t="str">
+        <x:v>Pass if all formatted strings match.</x:v>
+      </x:c>
+      <x:c r="H43" s="18" t="str">
+        <x:v>tests/test_regression.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="100" customHeight="1">
+      <x:c r="A44" s="18" t="str">
+        <x:v>UT-36</x:v>
+      </x:c>
+      <x:c r="B44" s="18" t="str">
+        <x:v>test_malformed_instructor_file_is_rejected</x:v>
+      </x:c>
+      <x:c r="C44" s="18" t="str">
+        <x:v>UC-02</x:v>
+      </x:c>
+      <x:c r="D44" s="18" t="str">
+        <x:v>Reject malformed instructor file.</x:v>
+      </x:c>
+      <x:c r="E44" s="18" t="str">
+        <x:v>programs/Test5.txt</x:v>
+      </x:c>
+      <x:c r="F44" s="18" t="str">
+        <x:v>ValueError.</x:v>
+      </x:c>
+      <x:c r="G44" s="18" t="str">
+        <x:v>Pass if load_program raises ValueError.</x:v>
+      </x:c>
+      <x:c r="H44" s="18" t="str">
+        <x:v>tests/test_regression.py</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52c4a821716546d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0897ad4c02fa4c93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>